<commit_message>
Add settings page and update templates with latest data.
Refresh car, sales, schedule pages and commit current project data JSON snapshots.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/uploads/배차관리_2025.xlsx
+++ b/uploads/배차관리_2025.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pdata\ojy-hmtaxi-erp\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5357458-BD7A-4AE9-9AF4-E64604885796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C7F52A-7DC7-42AF-B95A-4DD21962C7F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{66348461-5697-4C24-A8D1-6ED51936E14B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{66348461-5697-4C24-A8D1-6ED51936E14B}"/>
   </bookViews>
   <sheets>
     <sheet name="01월" sheetId="4" r:id="rId1"/>
@@ -24250,10 +24250,10 @@
       <c r="M1" s="3">
         <v>4</v>
       </c>
-      <c r="N1" s="3">
+      <c r="N1" s="8">
         <v>5</v>
       </c>
-      <c r="O1" s="8">
+      <c r="O1" s="3">
         <v>6</v>
       </c>
       <c r="P1" s="3">
@@ -24271,10 +24271,10 @@
       <c r="T1" s="3">
         <v>11</v>
       </c>
-      <c r="U1" s="3">
+      <c r="U1" s="8">
         <v>12</v>
       </c>
-      <c r="V1" s="8">
+      <c r="V1" s="3">
         <v>13</v>
       </c>
       <c r="W1" s="3">
@@ -24292,10 +24292,10 @@
       <c r="AA1" s="3">
         <v>18</v>
       </c>
-      <c r="AB1" s="3">
+      <c r="AB1" s="8">
         <v>19</v>
       </c>
-      <c r="AC1" s="8">
+      <c r="AC1" s="3">
         <v>20</v>
       </c>
       <c r="AD1" s="3">
@@ -24313,10 +24313,10 @@
       <c r="AH1" s="3">
         <v>25</v>
       </c>
-      <c r="AI1" s="3">
+      <c r="AI1" s="8">
         <v>26</v>
       </c>
-      <c r="AJ1" s="8">
+      <c r="AJ1" s="3">
         <v>27</v>
       </c>
       <c r="AK1" s="3">
@@ -24351,7 +24351,7 @@
       </c>
       <c r="G2" s="3">
         <f>COUNTIF(J2:AN2, "o")</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H2" s="3">
         <f>COUNTIF(J2:AN2, "x")</f>
@@ -24359,7 +24359,7 @@
       </c>
       <c r="I2" s="3">
         <f>SUM(COUNTIF(J2:AN2, "/"))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" s="7" t="s">
         <v>72</v>
@@ -24373,10 +24373,9 @@
       <c r="M2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O2" s="3"/>
+      <c r="O2" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P2" s="2" t="s">
         <v>72</v>
       </c>
@@ -24384,7 +24383,7 @@
         <v>72</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>72</v>
@@ -24392,10 +24391,9 @@
       <c r="T2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U2" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V2" s="3"/>
+      <c r="V2" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W2" s="2" t="s">
         <v>72</v>
       </c>
@@ -24411,10 +24409,9 @@
       <c r="AA2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB2" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC2" s="3"/>
+      <c r="AC2" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD2" s="2" t="s">
         <v>72</v>
       </c>
@@ -24430,10 +24427,9 @@
       <c r="AH2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI2" s="3" t="s">
+      <c r="AJ2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AJ2" s="3"/>
       <c r="AK2" s="2" t="s">
         <v>72</v>
       </c>
@@ -24462,19 +24458,19 @@
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F66" si="0">SUM(G3, I3, COUNTIF(J3:AN3, "H"))</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G66" si="1">COUNTIF(J3:AN3, "o")</f>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H3" s="3">
         <f t="shared" ref="H3:H66" si="2">COUNTIF(J3:AN3, "x")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" s="3">
         <f t="shared" ref="I3:I66" si="3">SUM(COUNTIF(J3:AN3, "/"))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>72</v>
@@ -24486,12 +24482,11 @@
         <v>72</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O3" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P3" s="2" t="s">
         <v>72</v>
       </c>
@@ -24507,10 +24502,9 @@
       <c r="T3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U3" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V3" s="3"/>
+      <c r="V3" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="W3" s="2" t="s">
         <v>72</v>
       </c>
@@ -24526,10 +24520,9 @@
       <c r="AA3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB3" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC3" s="3"/>
+      <c r="AC3" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD3" s="2" t="s">
         <v>72</v>
       </c>
@@ -24545,10 +24538,9 @@
       <c r="AH3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI3" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ3" s="3"/>
+      <c r="AJ3" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK3" s="2" t="s">
         <v>72</v>
       </c>
@@ -24603,10 +24595,9 @@
       <c r="M4" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="N4" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O4" s="3"/>
+      <c r="O4" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P4" s="2" t="s">
         <v>72</v>
       </c>
@@ -24622,10 +24613,9 @@
       <c r="T4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U4" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V4" s="3"/>
+      <c r="V4" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W4" s="2" t="s">
         <v>72</v>
       </c>
@@ -24641,10 +24631,9 @@
       <c r="AA4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC4" s="3"/>
+      <c r="AC4" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD4" s="2" t="s">
         <v>72</v>
       </c>
@@ -24660,10 +24649,9 @@
       <c r="AH4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI4" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ4" s="3"/>
+      <c r="AJ4" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK4" s="2" t="s">
         <v>72</v>
       </c>
@@ -24718,10 +24706,9 @@
       <c r="M5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="O5" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="O5" s="3"/>
       <c r="P5" s="2" t="s">
         <v>72</v>
       </c>
@@ -24737,10 +24724,9 @@
       <c r="T5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V5" s="3"/>
+      <c r="V5" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W5" s="2" t="s">
         <v>72</v>
       </c>
@@ -24756,10 +24742,9 @@
       <c r="AA5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC5" s="3"/>
+      <c r="AC5" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD5" s="2" t="s">
         <v>72</v>
       </c>
@@ -24775,10 +24760,9 @@
       <c r="AH5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI5" s="3" t="s">
+      <c r="AJ5" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AJ5" s="3"/>
       <c r="AK5" s="2" t="s">
         <v>72</v>
       </c>
@@ -24833,10 +24817,9 @@
       <c r="M6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="O6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="O6" s="3"/>
       <c r="P6" s="2" t="s">
         <v>72</v>
       </c>
@@ -24852,10 +24835,9 @@
       <c r="T6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U6" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V6" s="3"/>
+      <c r="V6" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W6" s="2" t="s">
         <v>72</v>
       </c>
@@ -24871,10 +24853,9 @@
       <c r="AA6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB6" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC6" s="3"/>
+      <c r="AC6" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD6" s="2" t="s">
         <v>72</v>
       </c>
@@ -24890,10 +24871,9 @@
       <c r="AH6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI6" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ6" s="3"/>
+      <c r="AJ6" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK6" s="2" t="s">
         <v>72</v>
       </c>
@@ -24948,10 +24928,9 @@
       <c r="M7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O7" s="3"/>
+      <c r="O7" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P7" s="2" t="s">
         <v>72</v>
       </c>
@@ -24967,10 +24946,9 @@
       <c r="T7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U7" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V7" s="3"/>
+      <c r="V7" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W7" s="2" t="s">
         <v>72</v>
       </c>
@@ -24986,10 +24964,9 @@
       <c r="AA7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB7" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC7" s="3"/>
+      <c r="AC7" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD7" s="2" t="s">
         <v>72</v>
       </c>
@@ -25005,10 +24982,9 @@
       <c r="AH7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI7" s="3" t="s">
+      <c r="AJ7" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AJ7" s="3"/>
       <c r="AK7" s="2" t="s">
         <v>72</v>
       </c>
@@ -25063,10 +25039,9 @@
       <c r="M8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N8" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O8" s="3"/>
+      <c r="O8" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P8" s="2" t="s">
         <v>72</v>
       </c>
@@ -25082,10 +25057,9 @@
       <c r="T8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U8" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V8" s="3"/>
+      <c r="V8" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W8" s="2" t="s">
         <v>72</v>
       </c>
@@ -25101,10 +25075,9 @@
       <c r="AA8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB8" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC8" s="3"/>
+      <c r="AC8" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD8" s="2" t="s">
         <v>72</v>
       </c>
@@ -25120,10 +25093,9 @@
       <c r="AH8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI8" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ8" s="3"/>
+      <c r="AJ8" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK8" s="2" t="s">
         <v>72</v>
       </c>
@@ -25178,10 +25150,9 @@
       <c r="M9" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="N9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O9" s="3"/>
+      <c r="O9" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P9" s="2" t="s">
         <v>72</v>
       </c>
@@ -25197,10 +25168,9 @@
       <c r="T9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V9" s="3"/>
+      <c r="V9" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W9" s="2" t="s">
         <v>72</v>
       </c>
@@ -25216,10 +25186,9 @@
       <c r="AA9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC9" s="3"/>
+      <c r="AC9" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD9" s="2" t="s">
         <v>72</v>
       </c>
@@ -25235,10 +25204,9 @@
       <c r="AH9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ9" s="3"/>
+      <c r="AJ9" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK9" s="2" t="s">
         <v>72</v>
       </c>
@@ -25293,10 +25261,9 @@
       <c r="M10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N10" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O10" s="3"/>
+      <c r="O10" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P10" s="2" t="s">
         <v>72</v>
       </c>
@@ -25312,10 +25279,9 @@
       <c r="T10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U10" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V10" s="3"/>
+      <c r="V10" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W10" s="2" t="s">
         <v>72</v>
       </c>
@@ -25331,10 +25297,9 @@
       <c r="AA10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB10" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC10" s="3"/>
+      <c r="AC10" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD10" s="2" t="s">
         <v>72</v>
       </c>
@@ -25350,10 +25315,9 @@
       <c r="AH10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI10" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ10" s="3"/>
+      <c r="AJ10" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK10" s="2" t="s">
         <v>72</v>
       </c>
@@ -25408,10 +25372,9 @@
       <c r="M11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N11" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O11" s="3"/>
+      <c r="O11" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P11" s="2" t="s">
         <v>72</v>
       </c>
@@ -25427,10 +25390,9 @@
       <c r="T11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U11" s="3" t="s">
+      <c r="V11" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="V11" s="3"/>
       <c r="W11" s="2" t="s">
         <v>77</v>
       </c>
@@ -25446,10 +25408,9 @@
       <c r="AA11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB11" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC11" s="3"/>
+      <c r="AC11" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD11" s="2" t="s">
         <v>72</v>
       </c>
@@ -25465,10 +25426,9 @@
       <c r="AH11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI11" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ11" s="3"/>
+      <c r="AJ11" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK11" s="2" t="s">
         <v>72</v>
       </c>
@@ -25523,10 +25483,9 @@
       <c r="M12" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O12" s="3"/>
+      <c r="O12" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P12" s="2" t="s">
         <v>72</v>
       </c>
@@ -25542,10 +25501,9 @@
       <c r="T12" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V12" s="3"/>
+      <c r="V12" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W12" s="2" t="s">
         <v>72</v>
       </c>
@@ -25561,10 +25519,9 @@
       <c r="AA12" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC12" s="3"/>
+      <c r="AC12" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD12" s="2" t="s">
         <v>72</v>
       </c>
@@ -25580,10 +25537,9 @@
       <c r="AH12" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ12" s="3"/>
+      <c r="AJ12" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK12" s="2" t="s">
         <v>72</v>
       </c>
@@ -25638,10 +25594,9 @@
       <c r="M13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N13" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O13" s="3"/>
+      <c r="O13" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P13" s="2" t="s">
         <v>72</v>
       </c>
@@ -25657,10 +25612,9 @@
       <c r="T13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U13" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V13" s="3"/>
+      <c r="V13" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W13" s="2" t="s">
         <v>72</v>
       </c>
@@ -25676,10 +25630,9 @@
       <c r="AA13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB13" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC13" s="3"/>
+      <c r="AC13" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD13" s="2" t="s">
         <v>72</v>
       </c>
@@ -25695,10 +25648,9 @@
       <c r="AH13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI13" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ13" s="3"/>
+      <c r="AJ13" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK13" s="2" t="s">
         <v>72</v>
       </c>
@@ -25753,10 +25705,9 @@
       <c r="M14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N14" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O14" s="3"/>
+      <c r="O14" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P14" s="2" t="s">
         <v>72</v>
       </c>
@@ -25772,10 +25723,9 @@
       <c r="T14" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="U14" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V14" s="3"/>
+      <c r="V14" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W14" s="2" t="s">
         <v>72</v>
       </c>
@@ -25791,10 +25741,9 @@
       <c r="AA14" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AB14" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC14" s="3"/>
+      <c r="AC14" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD14" s="2" t="s">
         <v>72</v>
       </c>
@@ -25810,10 +25759,9 @@
       <c r="AH14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI14" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ14" s="3"/>
+      <c r="AJ14" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK14" s="2" t="s">
         <v>72</v>
       </c>
@@ -25868,10 +25816,9 @@
       <c r="M15" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N15" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O15" s="3"/>
+      <c r="O15" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P15" s="2" t="s">
         <v>72</v>
       </c>
@@ -25887,10 +25834,9 @@
       <c r="T15" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U15" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V15" s="3"/>
+      <c r="V15" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W15" s="2" t="s">
         <v>72</v>
       </c>
@@ -25906,10 +25852,9 @@
       <c r="AA15" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB15" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC15" s="3"/>
+      <c r="AC15" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD15" s="2" t="s">
         <v>72</v>
       </c>
@@ -25925,10 +25870,9 @@
       <c r="AH15" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI15" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ15" s="3"/>
+      <c r="AJ15" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK15" s="2" t="s">
         <v>72</v>
       </c>
@@ -25983,10 +25927,9 @@
       <c r="M16" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="O16" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="O16" s="3"/>
       <c r="P16" s="2" t="s">
         <v>72</v>
       </c>
@@ -26002,10 +25945,9 @@
       <c r="T16" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U16" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V16" s="3"/>
+      <c r="V16" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W16" s="2" t="s">
         <v>72</v>
       </c>
@@ -26021,10 +25963,9 @@
       <c r="AA16" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB16" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC16" s="3"/>
+      <c r="AC16" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD16" s="2" t="s">
         <v>72</v>
       </c>
@@ -26040,10 +25981,9 @@
       <c r="AH16" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI16" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ16" s="3"/>
+      <c r="AJ16" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK16" s="7" t="s">
         <v>186</v>
       </c>
@@ -26098,10 +26038,9 @@
       <c r="M17" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N17" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O17" s="3"/>
+      <c r="O17" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P17" s="2" t="s">
         <v>72</v>
       </c>
@@ -26117,10 +26056,9 @@
       <c r="T17" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U17" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V17" s="3"/>
+      <c r="V17" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W17" s="2" t="s">
         <v>72</v>
       </c>
@@ -26136,10 +26074,9 @@
       <c r="AA17" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB17" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC17" s="3"/>
+      <c r="AC17" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD17" s="2" t="s">
         <v>72</v>
       </c>
@@ -26155,10 +26092,9 @@
       <c r="AH17" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI17" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ17" s="3"/>
+      <c r="AJ17" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK17" s="2" t="s">
         <v>72</v>
       </c>
@@ -26213,10 +26149,9 @@
       <c r="M18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N18" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O18" s="3"/>
+      <c r="O18" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P18" s="2" t="s">
         <v>72</v>
       </c>
@@ -26232,10 +26167,9 @@
       <c r="T18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U18" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V18" s="3"/>
+      <c r="V18" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W18" s="2" t="s">
         <v>72</v>
       </c>
@@ -26251,10 +26185,9 @@
       <c r="AA18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB18" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC18" s="3"/>
+      <c r="AC18" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD18" s="2" t="s">
         <v>72</v>
       </c>
@@ -26270,10 +26203,9 @@
       <c r="AH18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI18" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ18" s="3"/>
+      <c r="AJ18" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK18" s="2" t="s">
         <v>72</v>
       </c>
@@ -26328,10 +26260,9 @@
       <c r="M19" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N19" s="3" t="s">
+      <c r="O19" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="O19" s="3"/>
       <c r="P19" s="2" t="s">
         <v>72</v>
       </c>
@@ -26347,10 +26278,9 @@
       <c r="T19" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U19" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V19" s="3"/>
+      <c r="V19" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W19" s="2" t="s">
         <v>72</v>
       </c>
@@ -26366,10 +26296,9 @@
       <c r="AA19" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB19" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC19" s="3"/>
+      <c r="AC19" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD19" s="2" t="s">
         <v>72</v>
       </c>
@@ -26385,10 +26314,9 @@
       <c r="AH19" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI19" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ19" s="3"/>
+      <c r="AJ19" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK19" s="2" t="s">
         <v>72</v>
       </c>
@@ -26443,10 +26371,9 @@
       <c r="M20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O20" s="3"/>
+      <c r="O20" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P20" s="2" t="s">
         <v>72</v>
       </c>
@@ -26462,10 +26389,9 @@
       <c r="T20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V20" s="3"/>
+      <c r="V20" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W20" s="2" t="s">
         <v>72</v>
       </c>
@@ -26481,10 +26407,9 @@
       <c r="AA20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC20" s="3"/>
+      <c r="AC20" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD20" s="2" t="s">
         <v>72</v>
       </c>
@@ -26500,10 +26425,9 @@
       <c r="AH20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ20" s="3"/>
+      <c r="AJ20" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK20" s="2" t="s">
         <v>72</v>
       </c>
@@ -26558,10 +26482,9 @@
       <c r="M21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N21" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O21" s="3"/>
+      <c r="O21" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P21" s="2" t="s">
         <v>72</v>
       </c>
@@ -26577,10 +26500,9 @@
       <c r="T21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U21" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V21" s="3"/>
+      <c r="V21" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W21" s="2" t="s">
         <v>72</v>
       </c>
@@ -26596,10 +26518,9 @@
       <c r="AA21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB21" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC21" s="3"/>
+      <c r="AC21" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD21" s="2" t="s">
         <v>72</v>
       </c>
@@ -26615,10 +26536,9 @@
       <c r="AH21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI21" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ21" s="3"/>
+      <c r="AJ21" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK21" s="2" t="s">
         <v>72</v>
       </c>
@@ -26673,10 +26593,9 @@
       <c r="M22" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N22" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O22" s="3"/>
+      <c r="O22" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P22" s="2" t="s">
         <v>72</v>
       </c>
@@ -26692,10 +26611,9 @@
       <c r="T22" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U22" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V22" s="3"/>
+      <c r="V22" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W22" s="2" t="s">
         <v>72</v>
       </c>
@@ -26711,10 +26629,9 @@
       <c r="AA22" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB22" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC22" s="3"/>
+      <c r="AC22" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD22" s="2" t="s">
         <v>72</v>
       </c>
@@ -26730,10 +26647,9 @@
       <c r="AH22" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI22" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ22" s="3"/>
+      <c r="AJ22" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK22" s="2" t="s">
         <v>72</v>
       </c>
@@ -26788,10 +26704,9 @@
       <c r="M23" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N23" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O23" s="3"/>
+      <c r="O23" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P23" s="2" t="s">
         <v>72</v>
       </c>
@@ -26807,10 +26722,9 @@
       <c r="T23" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U23" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V23" s="3"/>
+      <c r="V23" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W23" s="2" t="s">
         <v>72</v>
       </c>
@@ -26826,10 +26740,9 @@
       <c r="AA23" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB23" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC23" s="3"/>
+      <c r="AC23" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD23" s="2" t="s">
         <v>72</v>
       </c>
@@ -26845,10 +26758,9 @@
       <c r="AH23" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI23" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ23" s="3"/>
+      <c r="AJ23" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK23" s="2" t="s">
         <v>72</v>
       </c>
@@ -26903,10 +26815,9 @@
       <c r="M24" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N24" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O24" s="3"/>
+      <c r="O24" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P24" s="2" t="s">
         <v>72</v>
       </c>
@@ -26922,10 +26833,9 @@
       <c r="T24" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U24" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V24" s="3"/>
+      <c r="V24" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W24" s="2" t="s">
         <v>72</v>
       </c>
@@ -26941,10 +26851,9 @@
       <c r="AA24" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB24" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC24" s="3"/>
+      <c r="AC24" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD24" s="2" t="s">
         <v>72</v>
       </c>
@@ -26960,10 +26869,9 @@
       <c r="AH24" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI24" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ24" s="3"/>
+      <c r="AJ24" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK24" s="2" t="s">
         <v>72</v>
       </c>
@@ -27018,10 +26926,9 @@
       <c r="M25" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O25" s="3"/>
+      <c r="O25" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P25" s="2" t="s">
         <v>72</v>
       </c>
@@ -27037,10 +26944,9 @@
       <c r="T25" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V25" s="3"/>
+      <c r="V25" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W25" s="2" t="s">
         <v>72</v>
       </c>
@@ -27056,10 +26962,9 @@
       <c r="AA25" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC25" s="3"/>
+      <c r="AC25" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD25" s="2" t="s">
         <v>72</v>
       </c>
@@ -27075,10 +26980,9 @@
       <c r="AH25" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ25" s="3"/>
+      <c r="AJ25" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK25" s="2" t="s">
         <v>72</v>
       </c>
@@ -27133,10 +27037,9 @@
       <c r="M26" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N26" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O26" s="3"/>
+      <c r="O26" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P26" s="2" t="s">
         <v>72</v>
       </c>
@@ -27152,10 +27055,9 @@
       <c r="T26" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U26" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V26" s="3"/>
+      <c r="V26" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W26" s="2" t="s">
         <v>72</v>
       </c>
@@ -27171,10 +27073,9 @@
       <c r="AA26" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB26" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC26" s="3"/>
+      <c r="AC26" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD26" s="2" t="s">
         <v>72</v>
       </c>
@@ -27190,10 +27091,9 @@
       <c r="AH26" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI26" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ26" s="3"/>
+      <c r="AJ26" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK26" s="2" t="s">
         <v>72</v>
       </c>
@@ -27248,10 +27148,9 @@
       <c r="M27" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N27" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O27" s="3"/>
+      <c r="O27" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P27" s="2" t="s">
         <v>72</v>
       </c>
@@ -27267,10 +27166,9 @@
       <c r="T27" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U27" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V27" s="3"/>
+      <c r="V27" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W27" s="2" t="s">
         <v>72</v>
       </c>
@@ -27286,10 +27184,9 @@
       <c r="AA27" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB27" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC27" s="3"/>
+      <c r="AC27" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD27" s="2" t="s">
         <v>72</v>
       </c>
@@ -27305,10 +27202,9 @@
       <c r="AH27" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI27" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ27" s="3"/>
+      <c r="AJ27" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK27" s="2" t="s">
         <v>72</v>
       </c>
@@ -27363,10 +27259,9 @@
       <c r="M28" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N28" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O28" s="3"/>
+      <c r="O28" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P28" s="2" t="s">
         <v>72</v>
       </c>
@@ -27382,10 +27277,9 @@
       <c r="T28" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U28" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V28" s="3"/>
+      <c r="V28" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W28" s="2" t="s">
         <v>72</v>
       </c>
@@ -27401,10 +27295,9 @@
       <c r="AA28" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB28" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC28" s="3"/>
+      <c r="AC28" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD28" s="2" t="s">
         <v>72</v>
       </c>
@@ -27420,10 +27313,9 @@
       <c r="AH28" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI28" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ28" s="3"/>
+      <c r="AJ28" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK28" s="2" t="s">
         <v>72</v>
       </c>
@@ -27478,10 +27370,9 @@
       <c r="M29" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N29" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O29" s="3"/>
+      <c r="O29" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P29" s="2" t="s">
         <v>72</v>
       </c>
@@ -27497,10 +27388,9 @@
       <c r="T29" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U29" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V29" s="3"/>
+      <c r="V29" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W29" s="2" t="s">
         <v>72</v>
       </c>
@@ -27516,10 +27406,9 @@
       <c r="AA29" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB29" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC29" s="3"/>
+      <c r="AC29" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD29" s="2" t="s">
         <v>72</v>
       </c>
@@ -27535,10 +27424,9 @@
       <c r="AH29" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI29" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ29" s="3"/>
+      <c r="AJ29" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK29" s="2" t="s">
         <v>72</v>
       </c>
@@ -27593,10 +27481,9 @@
       <c r="M30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N30" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O30" s="3"/>
+      <c r="O30" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P30" s="2" t="s">
         <v>72</v>
       </c>
@@ -27612,10 +27499,9 @@
       <c r="T30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U30" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V30" s="3"/>
+      <c r="V30" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W30" s="2" t="s">
         <v>72</v>
       </c>
@@ -27631,10 +27517,9 @@
       <c r="AA30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB30" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC30" s="3"/>
+      <c r="AC30" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD30" s="2" t="s">
         <v>72</v>
       </c>
@@ -27650,10 +27535,9 @@
       <c r="AH30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI30" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ30" s="3"/>
+      <c r="AJ30" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK30" s="2" t="s">
         <v>72</v>
       </c>
@@ -27708,10 +27592,9 @@
       <c r="M31" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N31" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O31" s="3"/>
+      <c r="O31" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P31" s="2" t="s">
         <v>72</v>
       </c>
@@ -27727,10 +27610,9 @@
       <c r="T31" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U31" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V31" s="3"/>
+      <c r="V31" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W31" s="2" t="s">
         <v>72</v>
       </c>
@@ -27746,10 +27628,9 @@
       <c r="AA31" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB31" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC31" s="3"/>
+      <c r="AC31" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD31" s="2" t="s">
         <v>72</v>
       </c>
@@ -27765,10 +27646,9 @@
       <c r="AH31" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI31" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ31" s="3"/>
+      <c r="AJ31" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK31" s="2" t="s">
         <v>72</v>
       </c>
@@ -27823,10 +27703,9 @@
       <c r="M32" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N32" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O32" s="3"/>
+      <c r="O32" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P32" s="2" t="s">
         <v>72</v>
       </c>
@@ -27842,10 +27721,9 @@
       <c r="T32" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U32" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V32" s="3"/>
+      <c r="V32" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W32" s="2" t="s">
         <v>72</v>
       </c>
@@ -27861,10 +27739,9 @@
       <c r="AA32" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB32" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC32" s="3"/>
+      <c r="AC32" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD32" s="2" t="s">
         <v>72</v>
       </c>
@@ -27880,10 +27757,9 @@
       <c r="AH32" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI32" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ32" s="3"/>
+      <c r="AJ32" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK32" s="2" t="s">
         <v>72</v>
       </c>
@@ -27938,10 +27814,9 @@
       <c r="M33" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N33" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O33" s="3"/>
+      <c r="O33" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P33" s="2" t="s">
         <v>72</v>
       </c>
@@ -27957,10 +27832,9 @@
       <c r="T33" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U33" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V33" s="3"/>
+      <c r="V33" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W33" s="2" t="s">
         <v>72</v>
       </c>
@@ -27976,10 +27850,9 @@
       <c r="AA33" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB33" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC33" s="3"/>
+      <c r="AC33" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD33" s="2" t="s">
         <v>72</v>
       </c>
@@ -27995,10 +27868,9 @@
       <c r="AH33" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI33" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ33" s="3"/>
+      <c r="AJ33" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK33" s="2" t="s">
         <v>72</v>
       </c>
@@ -28053,10 +27925,9 @@
       <c r="M34" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N34" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O34" s="3"/>
+      <c r="O34" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P34" s="2" t="s">
         <v>72</v>
       </c>
@@ -28072,10 +27943,9 @@
       <c r="T34" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U34" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V34" s="3"/>
+      <c r="V34" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W34" s="2" t="s">
         <v>72</v>
       </c>
@@ -28091,10 +27961,9 @@
       <c r="AA34" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB34" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC34" s="3"/>
+      <c r="AC34" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD34" s="2" t="s">
         <v>72</v>
       </c>
@@ -28110,10 +27979,9 @@
       <c r="AH34" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI34" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ34" s="3"/>
+      <c r="AJ34" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK34" s="2" t="s">
         <v>72</v>
       </c>
@@ -28168,10 +28036,9 @@
       <c r="M35" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N35" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O35" s="3"/>
+      <c r="O35" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P35" s="2" t="s">
         <v>72</v>
       </c>
@@ -28187,10 +28054,9 @@
       <c r="T35" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U35" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V35" s="3"/>
+      <c r="V35" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W35" s="2" t="s">
         <v>72</v>
       </c>
@@ -28206,10 +28072,9 @@
       <c r="AA35" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB35" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC35" s="3"/>
+      <c r="AC35" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD35" s="2" t="s">
         <v>72</v>
       </c>
@@ -28225,10 +28090,9 @@
       <c r="AH35" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI35" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ35" s="3"/>
+      <c r="AJ35" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK35" s="2" t="s">
         <v>72</v>
       </c>
@@ -28283,10 +28147,9 @@
       <c r="M36" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N36" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O36" s="3"/>
+      <c r="O36" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P36" s="2" t="s">
         <v>72</v>
       </c>
@@ -28302,10 +28165,9 @@
       <c r="T36" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U36" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V36" s="3"/>
+      <c r="V36" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W36" s="2" t="s">
         <v>72</v>
       </c>
@@ -28321,10 +28183,9 @@
       <c r="AA36" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB36" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC36" s="3"/>
+      <c r="AC36" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD36" s="2" t="s">
         <v>72</v>
       </c>
@@ -28340,10 +28201,9 @@
       <c r="AH36" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI36" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ36" s="3"/>
+      <c r="AJ36" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK36" s="2" t="s">
         <v>72</v>
       </c>
@@ -28398,10 +28258,9 @@
       <c r="M37" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N37" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O37" s="3"/>
+      <c r="O37" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P37" s="2" t="s">
         <v>72</v>
       </c>
@@ -28417,10 +28276,9 @@
       <c r="T37" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U37" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V37" s="3"/>
+      <c r="V37" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W37" s="2" t="s">
         <v>72</v>
       </c>
@@ -28436,10 +28294,9 @@
       <c r="AA37" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB37" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC37" s="3"/>
+      <c r="AC37" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD37" s="2" t="s">
         <v>72</v>
       </c>
@@ -28455,10 +28312,9 @@
       <c r="AH37" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI37" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ37" s="3"/>
+      <c r="AJ37" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK37" s="2" t="s">
         <v>72</v>
       </c>
@@ -28513,10 +28369,9 @@
       <c r="M38" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N38" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O38" s="3"/>
+      <c r="O38" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P38" s="2" t="s">
         <v>72</v>
       </c>
@@ -28532,10 +28387,9 @@
       <c r="T38" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U38" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V38" s="3"/>
+      <c r="V38" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W38" s="2" t="s">
         <v>72</v>
       </c>
@@ -28551,10 +28405,9 @@
       <c r="AA38" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB38" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC38" s="3"/>
+      <c r="AC38" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD38" s="2" t="s">
         <v>72</v>
       </c>
@@ -28570,10 +28423,9 @@
       <c r="AH38" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI38" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ38" s="3"/>
+      <c r="AJ38" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK38" s="2" t="s">
         <v>72</v>
       </c>
@@ -28628,10 +28480,9 @@
       <c r="M39" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N39" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O39" s="3"/>
+      <c r="O39" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P39" s="2" t="s">
         <v>72</v>
       </c>
@@ -28647,10 +28498,9 @@
       <c r="T39" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U39" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V39" s="3"/>
+      <c r="V39" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W39" s="2" t="s">
         <v>72</v>
       </c>
@@ -28666,10 +28516,9 @@
       <c r="AA39" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB39" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC39" s="3"/>
+      <c r="AC39" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD39" s="2" t="s">
         <v>72</v>
       </c>
@@ -28685,10 +28534,9 @@
       <c r="AH39" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI39" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ39" s="3"/>
+      <c r="AJ39" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK39" s="2" t="s">
         <v>72</v>
       </c>
@@ -28743,10 +28591,9 @@
       <c r="M40" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N40" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O40" s="3"/>
+      <c r="O40" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P40" s="2" t="s">
         <v>72</v>
       </c>
@@ -28762,10 +28609,9 @@
       <c r="T40" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U40" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V40" s="3"/>
+      <c r="V40" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W40" s="2" t="s">
         <v>72</v>
       </c>
@@ -28781,10 +28627,9 @@
       <c r="AA40" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB40" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC40" s="3"/>
+      <c r="AC40" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD40" s="2" t="s">
         <v>72</v>
       </c>
@@ -28800,10 +28645,9 @@
       <c r="AH40" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI40" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ40" s="3"/>
+      <c r="AJ40" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK40" s="2" t="s">
         <v>72</v>
       </c>
@@ -28858,10 +28702,9 @@
       <c r="M41" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N41" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O41" s="3"/>
+      <c r="O41" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P41" s="2" t="s">
         <v>72</v>
       </c>
@@ -28877,10 +28720,9 @@
       <c r="T41" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U41" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V41" s="3"/>
+      <c r="V41" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W41" s="2" t="s">
         <v>72</v>
       </c>
@@ -28896,10 +28738,9 @@
       <c r="AA41" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB41" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC41" s="3"/>
+      <c r="AC41" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD41" s="2" t="s">
         <v>72</v>
       </c>
@@ -28915,10 +28756,9 @@
       <c r="AH41" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI41" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ41" s="3"/>
+      <c r="AJ41" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK41" s="2" t="s">
         <v>72</v>
       </c>
@@ -28973,10 +28813,9 @@
       <c r="M42" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N42" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O42" s="3"/>
+      <c r="O42" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P42" s="2" t="s">
         <v>72</v>
       </c>
@@ -28992,10 +28831,9 @@
       <c r="T42" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U42" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V42" s="3"/>
+      <c r="V42" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W42" s="2" t="s">
         <v>72</v>
       </c>
@@ -29011,10 +28849,9 @@
       <c r="AA42" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB42" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC42" s="3"/>
+      <c r="AC42" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD42" s="2" t="s">
         <v>72</v>
       </c>
@@ -29030,10 +28867,9 @@
       <c r="AH42" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI42" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ42" s="3"/>
+      <c r="AJ42" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK42" s="2" t="s">
         <v>72</v>
       </c>
@@ -29088,10 +28924,9 @@
       <c r="M43" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N43" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O43" s="3"/>
+      <c r="O43" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P43" s="2" t="s">
         <v>72</v>
       </c>
@@ -29107,10 +28942,9 @@
       <c r="T43" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U43" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V43" s="3"/>
+      <c r="V43" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W43" s="2" t="s">
         <v>72</v>
       </c>
@@ -29126,10 +28960,9 @@
       <c r="AA43" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB43" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC43" s="3"/>
+      <c r="AC43" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD43" s="2" t="s">
         <v>72</v>
       </c>
@@ -29145,10 +28978,9 @@
       <c r="AH43" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI43" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ43" s="3"/>
+      <c r="AJ43" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK43" s="2" t="s">
         <v>72</v>
       </c>
@@ -29203,10 +29035,9 @@
       <c r="M44" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N44" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O44" s="3"/>
+      <c r="O44" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P44" s="2" t="s">
         <v>72</v>
       </c>
@@ -29222,10 +29053,9 @@
       <c r="T44" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U44" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V44" s="3"/>
+      <c r="V44" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W44" s="2" t="s">
         <v>72</v>
       </c>
@@ -29241,10 +29071,9 @@
       <c r="AA44" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB44" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC44" s="3"/>
+      <c r="AC44" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD44" s="2" t="s">
         <v>72</v>
       </c>
@@ -29260,10 +29089,9 @@
       <c r="AH44" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI44" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ44" s="3"/>
+      <c r="AJ44" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK44" s="2" t="s">
         <v>72</v>
       </c>
@@ -29318,10 +29146,9 @@
       <c r="M45" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N45" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O45" s="3"/>
+      <c r="O45" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P45" s="2" t="s">
         <v>72</v>
       </c>
@@ -29337,10 +29164,9 @@
       <c r="T45" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U45" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V45" s="3"/>
+      <c r="V45" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W45" s="2" t="s">
         <v>72</v>
       </c>
@@ -29356,10 +29182,9 @@
       <c r="AA45" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB45" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC45" s="3"/>
+      <c r="AC45" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD45" s="2" t="s">
         <v>72</v>
       </c>
@@ -29375,10 +29200,9 @@
       <c r="AH45" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI45" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ45" s="3"/>
+      <c r="AJ45" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK45" s="2" t="s">
         <v>72</v>
       </c>
@@ -29433,10 +29257,9 @@
       <c r="M46" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N46" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O46" s="3"/>
+      <c r="O46" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P46" s="2" t="s">
         <v>72</v>
       </c>
@@ -29452,10 +29275,9 @@
       <c r="T46" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U46" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V46" s="3"/>
+      <c r="V46" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W46" s="2" t="s">
         <v>72</v>
       </c>
@@ -29471,10 +29293,9 @@
       <c r="AA46" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB46" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC46" s="3"/>
+      <c r="AC46" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD46" s="2" t="s">
         <v>72</v>
       </c>
@@ -29490,10 +29311,9 @@
       <c r="AH46" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI46" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ46" s="3"/>
+      <c r="AJ46" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK46" s="2" t="s">
         <v>72</v>
       </c>
@@ -29548,10 +29368,9 @@
       <c r="M47" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N47" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O47" s="3"/>
+      <c r="O47" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P47" s="2" t="s">
         <v>72</v>
       </c>
@@ -29567,10 +29386,9 @@
       <c r="T47" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U47" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V47" s="3"/>
+      <c r="V47" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W47" s="2" t="s">
         <v>72</v>
       </c>
@@ -29586,10 +29404,9 @@
       <c r="AA47" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB47" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC47" s="3"/>
+      <c r="AC47" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD47" s="2" t="s">
         <v>72</v>
       </c>
@@ -29605,10 +29422,9 @@
       <c r="AH47" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI47" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ47" s="3"/>
+      <c r="AJ47" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK47" s="2" t="s">
         <v>72</v>
       </c>
@@ -29663,10 +29479,9 @@
       <c r="M48" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N48" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O48" s="3"/>
+      <c r="O48" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P48" s="2" t="s">
         <v>72</v>
       </c>
@@ -29682,10 +29497,9 @@
       <c r="T48" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U48" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V48" s="3"/>
+      <c r="V48" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W48" s="2" t="s">
         <v>72</v>
       </c>
@@ -29701,10 +29515,9 @@
       <c r="AA48" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB48" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC48" s="3"/>
+      <c r="AC48" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD48" s="2" t="s">
         <v>72</v>
       </c>
@@ -29720,10 +29533,9 @@
       <c r="AH48" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI48" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ48" s="3"/>
+      <c r="AJ48" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK48" s="2" t="s">
         <v>72</v>
       </c>
@@ -29778,10 +29590,9 @@
       <c r="M49" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N49" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O49" s="3"/>
+      <c r="O49" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P49" s="2" t="s">
         <v>72</v>
       </c>
@@ -29797,10 +29608,9 @@
       <c r="T49" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U49" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V49" s="3"/>
+      <c r="V49" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W49" s="2" t="s">
         <v>72</v>
       </c>
@@ -29816,10 +29626,9 @@
       <c r="AA49" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB49" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC49" s="3"/>
+      <c r="AC49" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD49" s="2" t="s">
         <v>72</v>
       </c>
@@ -29835,10 +29644,9 @@
       <c r="AH49" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI49" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ49" s="3"/>
+      <c r="AJ49" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK49" s="2" t="s">
         <v>72</v>
       </c>
@@ -29893,10 +29701,9 @@
       <c r="M50" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N50" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O50" s="3"/>
+      <c r="O50" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P50" s="2" t="s">
         <v>72</v>
       </c>
@@ -29912,10 +29719,9 @@
       <c r="T50" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U50" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V50" s="3"/>
+      <c r="V50" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W50" s="2" t="s">
         <v>72</v>
       </c>
@@ -29931,10 +29737,9 @@
       <c r="AA50" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB50" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC50" s="3"/>
+      <c r="AC50" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD50" s="2" t="s">
         <v>72</v>
       </c>
@@ -29950,10 +29755,9 @@
       <c r="AH50" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI50" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ50" s="3"/>
+      <c r="AJ50" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK50" s="2" t="s">
         <v>72</v>
       </c>
@@ -30008,10 +29812,9 @@
       <c r="M51" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N51" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O51" s="3"/>
+      <c r="O51" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P51" s="2" t="s">
         <v>72</v>
       </c>
@@ -30027,10 +29830,9 @@
       <c r="T51" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U51" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V51" s="3"/>
+      <c r="V51" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W51" s="2" t="s">
         <v>72</v>
       </c>
@@ -30046,10 +29848,9 @@
       <c r="AA51" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB51" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC51" s="3"/>
+      <c r="AC51" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD51" s="2" t="s">
         <v>72</v>
       </c>
@@ -30065,10 +29866,9 @@
       <c r="AH51" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI51" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ51" s="3"/>
+      <c r="AJ51" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK51" s="2" t="s">
         <v>72</v>
       </c>
@@ -30123,10 +29923,9 @@
       <c r="M52" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N52" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O52" s="3"/>
+      <c r="O52" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P52" s="2" t="s">
         <v>72</v>
       </c>
@@ -30142,10 +29941,9 @@
       <c r="T52" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U52" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V52" s="3"/>
+      <c r="V52" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W52" s="2" t="s">
         <v>72</v>
       </c>
@@ -30161,10 +29959,9 @@
       <c r="AA52" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB52" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC52" s="3"/>
+      <c r="AC52" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD52" s="2" t="s">
         <v>72</v>
       </c>
@@ -30180,10 +29977,9 @@
       <c r="AH52" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI52" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ52" s="3"/>
+      <c r="AJ52" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK52" s="2" t="s">
         <v>72</v>
       </c>
@@ -30238,10 +30034,9 @@
       <c r="M53" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N53" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O53" s="3"/>
+      <c r="O53" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P53" s="2" t="s">
         <v>72</v>
       </c>
@@ -30257,10 +30052,9 @@
       <c r="T53" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U53" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V53" s="3"/>
+      <c r="V53" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W53" s="2" t="s">
         <v>72</v>
       </c>
@@ -30276,10 +30070,9 @@
       <c r="AA53" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB53" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC53" s="3"/>
+      <c r="AC53" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD53" s="2" t="s">
         <v>72</v>
       </c>
@@ -30295,10 +30088,9 @@
       <c r="AH53" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI53" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ53" s="3"/>
+      <c r="AJ53" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK53" s="2" t="s">
         <v>72</v>
       </c>
@@ -30353,10 +30145,9 @@
       <c r="M54" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N54" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O54" s="3"/>
+      <c r="O54" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P54" s="2" t="s">
         <v>72</v>
       </c>
@@ -30372,10 +30163,9 @@
       <c r="T54" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U54" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V54" s="3"/>
+      <c r="V54" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W54" s="2" t="s">
         <v>72</v>
       </c>
@@ -30391,10 +30181,9 @@
       <c r="AA54" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB54" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC54" s="3"/>
+      <c r="AC54" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD54" s="2" t="s">
         <v>72</v>
       </c>
@@ -30410,10 +30199,9 @@
       <c r="AH54" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI54" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ54" s="3"/>
+      <c r="AJ54" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK54" s="2" t="s">
         <v>72</v>
       </c>
@@ -30468,10 +30256,9 @@
       <c r="M55" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N55" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O55" s="3"/>
+      <c r="O55" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P55" s="2" t="s">
         <v>72</v>
       </c>
@@ -30487,10 +30274,9 @@
       <c r="T55" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U55" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V55" s="3"/>
+      <c r="V55" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W55" s="2" t="s">
         <v>72</v>
       </c>
@@ -30506,10 +30292,9 @@
       <c r="AA55" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB55" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC55" s="3"/>
+      <c r="AC55" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD55" s="2" t="s">
         <v>72</v>
       </c>
@@ -30525,10 +30310,9 @@
       <c r="AH55" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI55" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ55" s="3"/>
+      <c r="AJ55" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK55" s="2" t="s">
         <v>72</v>
       </c>
@@ -30583,10 +30367,9 @@
       <c r="M56" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N56" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O56" s="3"/>
+      <c r="O56" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P56" s="2" t="s">
         <v>72</v>
       </c>
@@ -30602,10 +30385,9 @@
       <c r="T56" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U56" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V56" s="3"/>
+      <c r="V56" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W56" s="2" t="s">
         <v>72</v>
       </c>
@@ -30621,10 +30403,9 @@
       <c r="AA56" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB56" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC56" s="3"/>
+      <c r="AC56" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD56" s="2" t="s">
         <v>72</v>
       </c>
@@ -30640,10 +30421,9 @@
       <c r="AH56" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI56" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ56" s="3"/>
+      <c r="AJ56" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK56" s="2" t="s">
         <v>72</v>
       </c>
@@ -30698,10 +30478,9 @@
       <c r="M57" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N57" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O57" s="3"/>
+      <c r="O57" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P57" s="2" t="s">
         <v>72</v>
       </c>
@@ -30717,10 +30496,9 @@
       <c r="T57" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U57" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V57" s="3"/>
+      <c r="V57" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W57" s="2" t="s">
         <v>72</v>
       </c>
@@ -30736,10 +30514,9 @@
       <c r="AA57" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB57" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC57" s="3"/>
+      <c r="AC57" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD57" s="2" t="s">
         <v>72</v>
       </c>
@@ -30755,10 +30532,9 @@
       <c r="AH57" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI57" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ57" s="3"/>
+      <c r="AJ57" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK57" s="2" t="s">
         <v>72</v>
       </c>
@@ -30813,10 +30589,9 @@
       <c r="M58" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N58" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O58" s="3"/>
+      <c r="O58" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P58" s="2" t="s">
         <v>72</v>
       </c>
@@ -30832,10 +30607,9 @@
       <c r="T58" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U58" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V58" s="3"/>
+      <c r="V58" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W58" s="2" t="s">
         <v>72</v>
       </c>
@@ -30851,10 +30625,9 @@
       <c r="AA58" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB58" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC58" s="3"/>
+      <c r="AC58" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD58" s="2" t="s">
         <v>72</v>
       </c>
@@ -30870,10 +30643,9 @@
       <c r="AH58" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI58" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ58" s="3"/>
+      <c r="AJ58" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK58" s="2" t="s">
         <v>72</v>
       </c>
@@ -30928,10 +30700,9 @@
       <c r="M59" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N59" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O59" s="3"/>
+      <c r="O59" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P59" s="2" t="s">
         <v>72</v>
       </c>
@@ -30947,10 +30718,9 @@
       <c r="T59" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U59" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V59" s="3"/>
+      <c r="V59" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W59" s="2" t="s">
         <v>77</v>
       </c>
@@ -30966,10 +30736,9 @@
       <c r="AA59" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB59" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC59" s="3"/>
+      <c r="AC59" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD59" s="2" t="s">
         <v>72</v>
       </c>
@@ -30985,10 +30754,9 @@
       <c r="AH59" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI59" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ59" s="3"/>
+      <c r="AJ59" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK59" s="2" t="s">
         <v>72</v>
       </c>
@@ -31043,10 +30811,9 @@
       <c r="M60" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N60" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O60" s="3"/>
+      <c r="O60" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P60" s="2" t="s">
         <v>72</v>
       </c>
@@ -31062,10 +30829,9 @@
       <c r="T60" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U60" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V60" s="3"/>
+      <c r="V60" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W60" s="2" t="s">
         <v>72</v>
       </c>
@@ -31081,10 +30847,9 @@
       <c r="AA60" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB60" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC60" s="3"/>
+      <c r="AC60" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD60" s="2" t="s">
         <v>72</v>
       </c>
@@ -31100,10 +30865,9 @@
       <c r="AH60" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI60" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ60" s="3"/>
+      <c r="AJ60" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK60" s="2" t="s">
         <v>72</v>
       </c>
@@ -31158,10 +30922,9 @@
       <c r="M61" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N61" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O61" s="3"/>
+      <c r="O61" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P61" s="2" t="s">
         <v>72</v>
       </c>
@@ -31177,10 +30940,9 @@
       <c r="T61" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U61" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V61" s="3"/>
+      <c r="V61" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W61" s="2" t="s">
         <v>72</v>
       </c>
@@ -31196,10 +30958,9 @@
       <c r="AA61" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB61" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC61" s="3"/>
+      <c r="AC61" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD61" s="2" t="s">
         <v>72</v>
       </c>
@@ -31215,10 +30976,9 @@
       <c r="AH61" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI61" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ61" s="3"/>
+      <c r="AJ61" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK61" s="2" t="s">
         <v>72</v>
       </c>
@@ -31273,10 +31033,9 @@
       <c r="M62" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N62" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O62" s="3"/>
+      <c r="O62" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P62" s="2" t="s">
         <v>72</v>
       </c>
@@ -31292,10 +31051,9 @@
       <c r="T62" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U62" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V62" s="3"/>
+      <c r="V62" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W62" s="2" t="s">
         <v>72</v>
       </c>
@@ -31311,10 +31069,9 @@
       <c r="AA62" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB62" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC62" s="3"/>
+      <c r="AC62" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD62" s="2" t="s">
         <v>72</v>
       </c>
@@ -31330,10 +31087,9 @@
       <c r="AH62" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI62" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ62" s="3"/>
+      <c r="AJ62" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK62" s="2" t="s">
         <v>72</v>
       </c>
@@ -31388,10 +31144,9 @@
       <c r="M63" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N63" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O63" s="3"/>
+      <c r="O63" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P63" s="2" t="s">
         <v>72</v>
       </c>
@@ -31407,10 +31162,9 @@
       <c r="T63" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U63" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V63" s="3"/>
+      <c r="V63" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W63" s="2" t="s">
         <v>72</v>
       </c>
@@ -31426,10 +31180,9 @@
       <c r="AA63" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB63" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC63" s="3"/>
+      <c r="AC63" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD63" s="2" t="s">
         <v>72</v>
       </c>
@@ -31445,10 +31198,9 @@
       <c r="AH63" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI63" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ63" s="3"/>
+      <c r="AJ63" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK63" s="2" t="s">
         <v>72</v>
       </c>
@@ -31503,10 +31255,9 @@
       <c r="M64" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N64" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O64" s="3"/>
+      <c r="O64" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P64" s="2" t="s">
         <v>72</v>
       </c>
@@ -31522,10 +31273,9 @@
       <c r="T64" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U64" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V64" s="3"/>
+      <c r="V64" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W64" s="2" t="s">
         <v>72</v>
       </c>
@@ -31541,10 +31291,9 @@
       <c r="AA64" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB64" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC64" s="3"/>
+      <c r="AC64" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD64" s="2" t="s">
         <v>72</v>
       </c>
@@ -31560,10 +31309,9 @@
       <c r="AH64" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI64" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ64" s="3"/>
+      <c r="AJ64" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK64" s="2" t="s">
         <v>72</v>
       </c>
@@ -31618,10 +31366,9 @@
       <c r="M65" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N65" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O65" s="3"/>
+      <c r="O65" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P65" s="2" t="s">
         <v>72</v>
       </c>
@@ -31637,10 +31384,9 @@
       <c r="T65" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U65" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V65" s="3"/>
+      <c r="V65" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W65" s="2" t="s">
         <v>72</v>
       </c>
@@ -31656,10 +31402,9 @@
       <c r="AA65" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB65" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC65" s="3"/>
+      <c r="AC65" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD65" s="2" t="s">
         <v>72</v>
       </c>
@@ -31675,10 +31420,9 @@
       <c r="AH65" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI65" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ65" s="3"/>
+      <c r="AJ65" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK65" s="2" t="s">
         <v>72</v>
       </c>
@@ -31733,10 +31477,9 @@
       <c r="M66" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N66" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O66" s="3"/>
+      <c r="O66" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P66" s="2" t="s">
         <v>72</v>
       </c>
@@ -31752,10 +31495,9 @@
       <c r="T66" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U66" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V66" s="3"/>
+      <c r="V66" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W66" s="2" t="s">
         <v>72</v>
       </c>
@@ -31771,10 +31513,9 @@
       <c r="AA66" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB66" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC66" s="3"/>
+      <c r="AC66" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD66" s="2" t="s">
         <v>72</v>
       </c>
@@ -31790,10 +31531,9 @@
       <c r="AH66" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI66" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ66" s="3"/>
+      <c r="AJ66" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK66" s="2" t="s">
         <v>72</v>
       </c>
@@ -31848,10 +31588,9 @@
       <c r="M67" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N67" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O67" s="3"/>
+      <c r="O67" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P67" s="2" t="s">
         <v>72</v>
       </c>
@@ -31867,10 +31606,9 @@
       <c r="T67" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U67" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V67" s="3"/>
+      <c r="V67" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W67" s="2" t="s">
         <v>72</v>
       </c>
@@ -31886,10 +31624,9 @@
       <c r="AA67" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB67" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC67" s="3"/>
+      <c r="AC67" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD67" s="2" t="s">
         <v>72</v>
       </c>
@@ -31905,10 +31642,9 @@
       <c r="AH67" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI67" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ67" s="3"/>
+      <c r="AJ67" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK67" s="2" t="s">
         <v>72</v>
       </c>
@@ -31963,10 +31699,9 @@
       <c r="M68" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N68" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O68" s="3"/>
+      <c r="O68" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P68" s="2" t="s">
         <v>72</v>
       </c>
@@ -31982,10 +31717,9 @@
       <c r="T68" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U68" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V68" s="3"/>
+      <c r="V68" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W68" s="2" t="s">
         <v>72</v>
       </c>
@@ -32001,10 +31735,9 @@
       <c r="AA68" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB68" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC68" s="3"/>
+      <c r="AC68" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD68" s="2" t="s">
         <v>72</v>
       </c>
@@ -32020,10 +31753,9 @@
       <c r="AH68" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI68" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ68" s="3"/>
+      <c r="AJ68" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK68" s="2" t="s">
         <v>72</v>
       </c>
@@ -32078,10 +31810,9 @@
       <c r="M69" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N69" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O69" s="3"/>
+      <c r="O69" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P69" s="2" t="s">
         <v>72</v>
       </c>
@@ -32097,10 +31828,9 @@
       <c r="T69" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U69" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V69" s="3"/>
+      <c r="V69" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W69" s="2" t="s">
         <v>72</v>
       </c>
@@ -32116,10 +31846,9 @@
       <c r="AA69" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB69" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC69" s="3"/>
+      <c r="AC69" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD69" s="2" t="s">
         <v>72</v>
       </c>
@@ -32135,10 +31864,9 @@
       <c r="AH69" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI69" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ69" s="3"/>
+      <c r="AJ69" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK69" s="2" t="s">
         <v>72</v>
       </c>
@@ -32193,10 +31921,9 @@
       <c r="M70" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N70" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O70" s="3"/>
+      <c r="O70" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P70" s="2" t="s">
         <v>72</v>
       </c>
@@ -32212,10 +31939,9 @@
       <c r="T70" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U70" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V70" s="3"/>
+      <c r="V70" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W70" s="2" t="s">
         <v>72</v>
       </c>
@@ -32231,10 +31957,9 @@
       <c r="AA70" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB70" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC70" s="3"/>
+      <c r="AC70" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD70" s="2" t="s">
         <v>72</v>
       </c>
@@ -32250,10 +31975,9 @@
       <c r="AH70" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI70" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ70" s="3"/>
+      <c r="AJ70" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK70" s="2" t="s">
         <v>72</v>
       </c>
@@ -32308,10 +32032,9 @@
       <c r="M71" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N71" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O71" s="3"/>
+      <c r="O71" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P71" s="2" t="s">
         <v>72</v>
       </c>
@@ -32327,10 +32050,9 @@
       <c r="T71" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U71" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V71" s="3"/>
+      <c r="V71" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W71" s="2" t="s">
         <v>72</v>
       </c>
@@ -32346,10 +32068,9 @@
       <c r="AA71" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB71" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC71" s="3"/>
+      <c r="AC71" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD71" s="2" t="s">
         <v>72</v>
       </c>
@@ -32365,10 +32086,9 @@
       <c r="AH71" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI71" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ71" s="3"/>
+      <c r="AJ71" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK71" s="2" t="s">
         <v>72</v>
       </c>
@@ -32423,10 +32143,9 @@
       <c r="M72" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N72" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O72" s="3"/>
+      <c r="O72" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P72" s="2" t="s">
         <v>72</v>
       </c>
@@ -32442,10 +32161,9 @@
       <c r="T72" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U72" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V72" s="3"/>
+      <c r="V72" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W72" s="2" t="s">
         <v>72</v>
       </c>
@@ -32461,10 +32179,9 @@
       <c r="AA72" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB72" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC72" s="3"/>
+      <c r="AC72" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD72" s="2" t="s">
         <v>72</v>
       </c>
@@ -32480,10 +32197,9 @@
       <c r="AH72" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI72" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ72" s="3"/>
+      <c r="AJ72" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK72" s="2" t="s">
         <v>72</v>
       </c>
@@ -32538,10 +32254,9 @@
       <c r="M73" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N73" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O73" s="3"/>
+      <c r="O73" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P73" s="2" t="s">
         <v>72</v>
       </c>
@@ -32557,10 +32272,9 @@
       <c r="T73" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U73" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V73" s="3"/>
+      <c r="V73" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W73" s="2" t="s">
         <v>72</v>
       </c>
@@ -32576,10 +32290,9 @@
       <c r="AA73" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB73" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC73" s="3"/>
+      <c r="AC73" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD73" s="2" t="s">
         <v>72</v>
       </c>
@@ -32595,10 +32308,9 @@
       <c r="AH73" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI73" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ73" s="3"/>
+      <c r="AJ73" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK73" s="2" t="s">
         <v>72</v>
       </c>
@@ -32653,10 +32365,9 @@
       <c r="M74" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N74" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O74" s="3"/>
+      <c r="O74" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P74" s="2" t="s">
         <v>72</v>
       </c>
@@ -32672,10 +32383,9 @@
       <c r="T74" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U74" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V74" s="3"/>
+      <c r="V74" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W74" s="2" t="s">
         <v>72</v>
       </c>
@@ -32691,10 +32401,9 @@
       <c r="AA74" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB74" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC74" s="3"/>
+      <c r="AC74" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD74" s="2" t="s">
         <v>72</v>
       </c>
@@ -32710,10 +32419,9 @@
       <c r="AH74" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI74" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ74" s="3"/>
+      <c r="AJ74" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK74" s="2" t="s">
         <v>72</v>
       </c>
@@ -32768,10 +32476,9 @@
       <c r="M75" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N75" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O75" s="3"/>
+      <c r="O75" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P75" s="2" t="s">
         <v>72</v>
       </c>
@@ -32787,10 +32494,9 @@
       <c r="T75" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U75" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V75" s="3"/>
+      <c r="V75" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W75" s="2" t="s">
         <v>72</v>
       </c>
@@ -32806,10 +32512,9 @@
       <c r="AA75" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB75" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC75" s="3"/>
+      <c r="AC75" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD75" s="2" t="s">
         <v>72</v>
       </c>
@@ -32825,10 +32530,9 @@
       <c r="AH75" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI75" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ75" s="3"/>
+      <c r="AJ75" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK75" s="2" t="s">
         <v>72</v>
       </c>
@@ -32883,10 +32587,9 @@
       <c r="M76" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N76" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O76" s="3"/>
+      <c r="O76" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P76" s="2" t="s">
         <v>72</v>
       </c>
@@ -32902,10 +32605,9 @@
       <c r="T76" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U76" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V76" s="3"/>
+      <c r="V76" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W76" s="2" t="s">
         <v>72</v>
       </c>
@@ -32921,10 +32623,9 @@
       <c r="AA76" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB76" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC76" s="3"/>
+      <c r="AC76" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD76" s="2" t="s">
         <v>72</v>
       </c>
@@ -32940,10 +32641,9 @@
       <c r="AH76" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI76" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ76" s="3"/>
+      <c r="AJ76" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK76" s="2" t="s">
         <v>72</v>
       </c>
@@ -32998,10 +32698,9 @@
       <c r="M77" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N77" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O77" s="3"/>
+      <c r="O77" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P77" s="2" t="s">
         <v>72</v>
       </c>
@@ -33017,10 +32716,9 @@
       <c r="T77" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U77" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V77" s="3"/>
+      <c r="V77" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W77" s="2" t="s">
         <v>72</v>
       </c>
@@ -33036,10 +32734,9 @@
       <c r="AA77" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB77" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC77" s="3"/>
+      <c r="AC77" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD77" s="2" t="s">
         <v>72</v>
       </c>
@@ -33055,10 +32752,9 @@
       <c r="AH77" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI77" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ77" s="3"/>
+      <c r="AJ77" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK77" s="2" t="s">
         <v>72</v>
       </c>
@@ -33113,10 +32809,9 @@
       <c r="M78" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N78" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O78" s="3"/>
+      <c r="O78" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P78" s="2" t="s">
         <v>72</v>
       </c>
@@ -33132,10 +32827,9 @@
       <c r="T78" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U78" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V78" s="3"/>
+      <c r="V78" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W78" s="2" t="s">
         <v>72</v>
       </c>
@@ -33151,10 +32845,9 @@
       <c r="AA78" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB78" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC78" s="3"/>
+      <c r="AC78" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD78" s="2" t="s">
         <v>72</v>
       </c>
@@ -33170,10 +32863,9 @@
       <c r="AH78" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI78" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ78" s="3"/>
+      <c r="AJ78" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK78" s="2" t="s">
         <v>72</v>
       </c>
@@ -33228,10 +32920,9 @@
       <c r="M79" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N79" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O79" s="3"/>
+      <c r="O79" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P79" s="2" t="s">
         <v>72</v>
       </c>
@@ -33247,10 +32938,9 @@
       <c r="T79" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U79" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V79" s="3"/>
+      <c r="V79" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W79" s="2" t="s">
         <v>72</v>
       </c>
@@ -33266,10 +32956,9 @@
       <c r="AA79" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB79" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC79" s="3"/>
+      <c r="AC79" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD79" s="2" t="s">
         <v>72</v>
       </c>
@@ -33285,10 +32974,9 @@
       <c r="AH79" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI79" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ79" s="3"/>
+      <c r="AJ79" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK79" s="2" t="s">
         <v>72</v>
       </c>
@@ -33329,28 +33017,24 @@
       <c r="K80" s="3"/>
       <c r="L80" s="3"/>
       <c r="M80" s="3"/>
-      <c r="N80" s="3"/>
       <c r="O80" s="3"/>
       <c r="P80" s="2"/>
       <c r="Q80" s="3"/>
       <c r="R80" s="3"/>
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
-      <c r="U80" s="3"/>
       <c r="V80" s="3"/>
       <c r="W80" s="2"/>
       <c r="X80" s="3"/>
       <c r="Y80" s="3"/>
       <c r="Z80" s="3"/>
       <c r="AA80" s="3"/>
-      <c r="AB80" s="3"/>
       <c r="AC80" s="3"/>
       <c r="AD80" s="2"/>
       <c r="AE80" s="3"/>
       <c r="AF80" s="3"/>
       <c r="AG80" s="3"/>
       <c r="AH80" s="3"/>
-      <c r="AI80" s="3"/>
       <c r="AJ80" s="3"/>
       <c r="AK80" s="2"/>
       <c r="AL80" s="3"/>
@@ -33386,28 +33070,24 @@
       <c r="K81" s="3"/>
       <c r="L81" s="3"/>
       <c r="M81" s="3"/>
-      <c r="N81" s="3"/>
       <c r="O81" s="3"/>
       <c r="P81" s="2"/>
       <c r="Q81" s="3"/>
       <c r="R81" s="3"/>
       <c r="S81" s="3"/>
       <c r="T81" s="3"/>
-      <c r="U81" s="3"/>
       <c r="V81" s="3"/>
       <c r="W81" s="2"/>
       <c r="X81" s="3"/>
       <c r="Y81" s="3"/>
       <c r="Z81" s="3"/>
       <c r="AA81" s="3"/>
-      <c r="AB81" s="3"/>
       <c r="AC81" s="3"/>
       <c r="AD81" s="2"/>
       <c r="AE81" s="3"/>
       <c r="AF81" s="3"/>
       <c r="AG81" s="3"/>
       <c r="AH81" s="3"/>
-      <c r="AI81" s="3"/>
       <c r="AJ81" s="3"/>
       <c r="AK81" s="2"/>
       <c r="AL81" s="3"/>
@@ -33457,10 +33137,9 @@
       <c r="M82" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N82" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O82" s="3"/>
+      <c r="O82" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P82" s="2" t="s">
         <v>72</v>
       </c>
@@ -33476,10 +33155,9 @@
       <c r="T82" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U82" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V82" s="3"/>
+      <c r="V82" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W82" s="2" t="s">
         <v>72</v>
       </c>
@@ -33495,10 +33173,9 @@
       <c r="AA82" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB82" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC82" s="3"/>
+      <c r="AC82" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD82" s="2" t="s">
         <v>72</v>
       </c>
@@ -33514,10 +33191,9 @@
       <c r="AH82" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI82" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ82" s="3"/>
+      <c r="AJ82" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK82" s="2" t="s">
         <v>72</v>
       </c>
@@ -33572,10 +33248,9 @@
       <c r="M83" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N83" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O83" s="3"/>
+      <c r="O83" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P83" s="2" t="s">
         <v>72</v>
       </c>
@@ -33591,10 +33266,9 @@
       <c r="T83" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U83" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V83" s="3"/>
+      <c r="V83" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W83" s="2" t="s">
         <v>72</v>
       </c>
@@ -33610,10 +33284,9 @@
       <c r="AA83" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB83" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC83" s="3"/>
+      <c r="AC83" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD83" s="2" t="s">
         <v>72</v>
       </c>
@@ -33629,10 +33302,9 @@
       <c r="AH83" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI83" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ83" s="3"/>
+      <c r="AJ83" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK83" s="2" t="s">
         <v>72</v>
       </c>
@@ -33687,10 +33359,9 @@
       <c r="M84" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N84" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O84" s="3"/>
+      <c r="O84" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P84" s="2" t="s">
         <v>72</v>
       </c>
@@ -33706,10 +33377,9 @@
       <c r="T84" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U84" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V84" s="3"/>
+      <c r="V84" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W84" s="2" t="s">
         <v>72</v>
       </c>
@@ -33725,10 +33395,9 @@
       <c r="AA84" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB84" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC84" s="3"/>
+      <c r="AC84" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD84" s="2" t="s">
         <v>72</v>
       </c>
@@ -33744,10 +33413,9 @@
       <c r="AH84" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI84" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ84" s="3"/>
+      <c r="AJ84" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK84" s="2" t="s">
         <v>72</v>
       </c>
@@ -33802,10 +33470,9 @@
       <c r="M85" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N85" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O85" s="3"/>
+      <c r="O85" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P85" s="2" t="s">
         <v>72</v>
       </c>
@@ -33821,10 +33488,9 @@
       <c r="T85" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U85" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V85" s="3"/>
+      <c r="V85" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W85" s="2" t="s">
         <v>72</v>
       </c>
@@ -33840,10 +33506,9 @@
       <c r="AA85" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB85" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC85" s="3"/>
+      <c r="AC85" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD85" s="2" t="s">
         <v>72</v>
       </c>
@@ -33859,10 +33524,9 @@
       <c r="AH85" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI85" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ85" s="3"/>
+      <c r="AJ85" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK85" s="2" t="s">
         <v>72</v>
       </c>
@@ -33917,10 +33581,9 @@
       <c r="M86" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N86" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O86" s="3"/>
+      <c r="O86" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P86" s="2" t="s">
         <v>72</v>
       </c>
@@ -33936,10 +33599,9 @@
       <c r="T86" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U86" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V86" s="3"/>
+      <c r="V86" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W86" s="2" t="s">
         <v>72</v>
       </c>
@@ -33955,10 +33617,9 @@
       <c r="AA86" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB86" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC86" s="3"/>
+      <c r="AC86" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD86" s="2" t="s">
         <v>72</v>
       </c>
@@ -33974,10 +33635,9 @@
       <c r="AH86" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI86" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ86" s="3"/>
+      <c r="AJ86" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK86" s="2" t="s">
         <v>72</v>
       </c>
@@ -34032,10 +33692,9 @@
       <c r="M87" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N87" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O87" s="3"/>
+      <c r="O87" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P87" s="2" t="s">
         <v>72</v>
       </c>
@@ -34051,10 +33710,9 @@
       <c r="T87" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U87" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V87" s="3"/>
+      <c r="V87" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W87" s="2" t="s">
         <v>72</v>
       </c>
@@ -34070,10 +33728,9 @@
       <c r="AA87" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB87" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC87" s="3"/>
+      <c r="AC87" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD87" s="2" t="s">
         <v>72</v>
       </c>
@@ -34089,10 +33746,9 @@
       <c r="AH87" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI87" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ87" s="3"/>
+      <c r="AJ87" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK87" s="2" t="s">
         <v>72</v>
       </c>
@@ -34147,10 +33803,9 @@
       <c r="M88" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N88" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O88" s="3"/>
+      <c r="O88" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P88" s="2" t="s">
         <v>72</v>
       </c>
@@ -34166,10 +33821,9 @@
       <c r="T88" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U88" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V88" s="3"/>
+      <c r="V88" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W88" s="2" t="s">
         <v>72</v>
       </c>
@@ -34185,10 +33839,9 @@
       <c r="AA88" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB88" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC88" s="3"/>
+      <c r="AC88" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD88" s="2" t="s">
         <v>72</v>
       </c>
@@ -34204,10 +33857,9 @@
       <c r="AH88" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI88" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ88" s="3"/>
+      <c r="AJ88" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK88" s="2" t="s">
         <v>72</v>
       </c>
@@ -34262,10 +33914,9 @@
       <c r="M89" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N89" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O89" s="3"/>
+      <c r="O89" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P89" s="2" t="s">
         <v>72</v>
       </c>
@@ -34281,10 +33932,9 @@
       <c r="T89" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="U89" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="V89" s="3"/>
+      <c r="V89" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="W89" s="2" t="s">
         <v>72</v>
       </c>
@@ -34300,10 +33950,9 @@
       <c r="AA89" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB89" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC89" s="3"/>
+      <c r="AC89" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AD89" s="2" t="s">
         <v>72</v>
       </c>
@@ -34319,10 +33968,9 @@
       <c r="AH89" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AI89" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ89" s="3"/>
+      <c r="AJ89" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AK89" s="2" t="s">
         <v>72</v>
       </c>
@@ -34352,7 +34000,7 @@
       <formula>NOT(ISERROR(SEARCH("주간",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:AM1048576">
+  <conditionalFormatting sqref="J1:AM1 J2:M89 O2:T89 V2:AA89 AC2:AH89 AJ2:AM89 J90:AM1048576">
     <cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="R">
       <formula>NOT(ISERROR(SEARCH("R",J1)))</formula>
     </cfRule>

</xml_diff>